<commit_message>
Resolve genus-level taxa and update species lookup
</commit_message>
<xml_diff>
--- a/data/processed/unique_species_lookup_edited.xlsx
+++ b/data/processed/unique_species_lookup_edited.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/44e88a4787a5f5bb/Desktop/TURF_DATA/species_lookups/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/44e88a4787a5f5bb/Desktop/TURF_DATA/mex-TURFs-main/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{0E14D389-A550-4F69-B427-5429ABA35EC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BF66311-316E-4428-BE84-E775647AEE6F}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="8_{0E14D389-A550-4F69-B427-5429ABA35EC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BCAE6CA-0DE0-461B-A6C4-2FF727588DC8}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{7358565B-5D53-4AC9-BDCB-AD95EAEBAD41}"/>
+    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{7358565B-5D53-4AC9-BDCB-AD95EAEBAD41}"/>
   </bookViews>
   <sheets>
     <sheet name="species_lookup" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="284">
   <si>
     <t>turf_id</t>
   </si>
@@ -82,784 +82,796 @@
     <t>Crassostrea virginica</t>
   </si>
   <si>
+    <t>MX_C_196</t>
+  </si>
+  <si>
+    <t>MX_C_193</t>
+  </si>
+  <si>
+    <t>MX_C_203</t>
+  </si>
+  <si>
+    <t>MX_C_209</t>
+  </si>
+  <si>
+    <t>MX_C_205</t>
+  </si>
+  <si>
+    <t>MX_C_052</t>
+  </si>
+  <si>
+    <t>Gelidium</t>
+  </si>
+  <si>
+    <t>ALGAS MARINAS</t>
+  </si>
+  <si>
+    <t>MX_C_007</t>
+  </si>
+  <si>
+    <t>Gelidium robustum</t>
+  </si>
+  <si>
+    <t>SARGAZO ROJO</t>
+  </si>
+  <si>
+    <t>MX_C_018</t>
+  </si>
+  <si>
+    <t>MX_C_031</t>
+  </si>
+  <si>
+    <t>MX_C_032</t>
+  </si>
+  <si>
+    <t>MX_C_024</t>
+  </si>
+  <si>
+    <t>Haliotis corrugata</t>
+  </si>
+  <si>
+    <t>ABULON AMARILLO</t>
+  </si>
+  <si>
+    <t>ABULON AZUL</t>
+  </si>
+  <si>
+    <t>MX_C_009</t>
+  </si>
+  <si>
+    <t>ABULON</t>
+  </si>
+  <si>
+    <t>MX_C_025</t>
+  </si>
+  <si>
+    <t>MX_C_029</t>
+  </si>
+  <si>
+    <t>MX_C_041</t>
+  </si>
+  <si>
+    <t>CAMARON AZUL</t>
+  </si>
+  <si>
+    <t>MX_C_037</t>
+  </si>
+  <si>
+    <t>MX_C_003</t>
+  </si>
+  <si>
+    <t>MX_C_051</t>
+  </si>
+  <si>
+    <t>MX_C_047</t>
+  </si>
+  <si>
+    <t>Macrobrachium carcinus</t>
+  </si>
+  <si>
+    <t>LANGOSTINO</t>
+  </si>
+  <si>
+    <t>ACAMAYA</t>
+  </si>
+  <si>
+    <t>CARACOL BURRO</t>
+  </si>
+  <si>
+    <t>LANGOSTA ROJA</t>
+  </si>
+  <si>
+    <t>MX_C_066</t>
+  </si>
+  <si>
+    <t>Panulirus argus</t>
+  </si>
+  <si>
+    <t>LANGOSTA DEL CARIBE</t>
+  </si>
+  <si>
+    <t>MX_C_065</t>
+  </si>
+  <si>
+    <t>MX_C_068</t>
+  </si>
+  <si>
+    <t>MX_C_067</t>
+  </si>
+  <si>
+    <t>MX_C_064</t>
+  </si>
+  <si>
+    <t>MX_C_063</t>
+  </si>
+  <si>
+    <t>MX_C_062</t>
+  </si>
+  <si>
+    <t>MX_C_061</t>
+  </si>
+  <si>
+    <t>MX_C_217</t>
+  </si>
+  <si>
+    <t>MX_C_216</t>
+  </si>
+  <si>
+    <t>MX_C_215</t>
+  </si>
+  <si>
+    <t>MX_C_214</t>
+  </si>
+  <si>
+    <t>MX_C_213</t>
+  </si>
+  <si>
+    <t>Panulirus gracilis</t>
+  </si>
+  <si>
+    <t>LANGOSTA VERDE</t>
+  </si>
+  <si>
+    <t>Panulirus inflatus</t>
+  </si>
+  <si>
+    <t>LANGOSTA AZUL</t>
+  </si>
+  <si>
+    <t>Panulirus spp.</t>
+  </si>
+  <si>
+    <t>LANGOSTA</t>
+  </si>
+  <si>
+    <t>Penaeus aztecus</t>
+  </si>
+  <si>
+    <t>CAMARON CAFE</t>
+  </si>
+  <si>
+    <t>MX_C_039</t>
+  </si>
+  <si>
+    <t>MX_C_002</t>
+  </si>
+  <si>
+    <t>Penaeus spp.</t>
+  </si>
+  <si>
+    <t>CAMARON DE ESTERO</t>
+  </si>
+  <si>
+    <t>MX_C_057</t>
+  </si>
+  <si>
+    <t>MX_C_046</t>
+  </si>
+  <si>
+    <t>MX_C_045</t>
+  </si>
+  <si>
+    <t>MX_C_044</t>
+  </si>
+  <si>
+    <t>MX_C_043</t>
+  </si>
+  <si>
+    <t>MX_C_004</t>
+  </si>
+  <si>
+    <t>MX_C_055</t>
+  </si>
+  <si>
+    <t>MX_C_036</t>
+  </si>
+  <si>
+    <t>MX_C_035</t>
+  </si>
+  <si>
+    <t>MX_C_034</t>
+  </si>
+  <si>
+    <t>MX_C_033</t>
+  </si>
+  <si>
+    <t>MX_C_040</t>
+  </si>
+  <si>
+    <t>MX_C_054</t>
+  </si>
+  <si>
+    <t>MX_C_050</t>
+  </si>
+  <si>
+    <t>MX_C_098</t>
+  </si>
+  <si>
+    <t>MX_C_089</t>
+  </si>
+  <si>
+    <t>MX_C_088</t>
+  </si>
+  <si>
+    <t>MX_C_086</t>
+  </si>
+  <si>
+    <t>MX_C_085</t>
+  </si>
+  <si>
+    <t>MX_C_083</t>
+  </si>
+  <si>
+    <t>MX_C_082</t>
+  </si>
+  <si>
+    <t>MX_C_081</t>
+  </si>
+  <si>
+    <t>MX_C_080</t>
+  </si>
+  <si>
+    <t>MX_C_078</t>
+  </si>
+  <si>
+    <t>MX_C_097</t>
+  </si>
+  <si>
+    <t>MX_C_076</t>
+  </si>
+  <si>
+    <t>MX_C_075</t>
+  </si>
+  <si>
+    <t>MX_C_074</t>
+  </si>
+  <si>
+    <t>MX_C_073</t>
+  </si>
+  <si>
+    <t>MX_C_072</t>
+  </si>
+  <si>
+    <t>MX_C_071</t>
+  </si>
+  <si>
+    <t>MX_C_070</t>
+  </si>
+  <si>
+    <t>MX_C_069</t>
+  </si>
+  <si>
+    <t>MX_C_189</t>
+  </si>
+  <si>
+    <t>MX_C_188</t>
+  </si>
+  <si>
+    <t>MX_C_096</t>
+  </si>
+  <si>
+    <t>MX_C_187</t>
+  </si>
+  <si>
+    <t>MX_C_186</t>
+  </si>
+  <si>
+    <t>MX_C_185</t>
+  </si>
+  <si>
+    <t>MX_C_184</t>
+  </si>
+  <si>
+    <t>MX_C_183</t>
+  </si>
+  <si>
+    <t>MX_C_182</t>
+  </si>
+  <si>
+    <t>MX_C_181</t>
+  </si>
+  <si>
+    <t>MX_C_180</t>
+  </si>
+  <si>
+    <t>MX_C_179</t>
+  </si>
+  <si>
+    <t>MX_C_178</t>
+  </si>
+  <si>
+    <t>MX_C_095</t>
+  </si>
+  <si>
+    <t>MX_C_177</t>
+  </si>
+  <si>
+    <t>MX_C_176</t>
+  </si>
+  <si>
+    <t>MX_C_175</t>
+  </si>
+  <si>
+    <t>MX_C_174</t>
+  </si>
+  <si>
+    <t>MX_C_173</t>
+  </si>
+  <si>
+    <t>MX_C_172</t>
+  </si>
+  <si>
+    <t>MX_C_171</t>
+  </si>
+  <si>
+    <t>MX_C_170</t>
+  </si>
+  <si>
+    <t>MX_C_169</t>
+  </si>
+  <si>
+    <t>MX_C_168</t>
+  </si>
+  <si>
+    <t>MX_C_094</t>
+  </si>
+  <si>
+    <t>MX_C_167</t>
+  </si>
+  <si>
+    <t>MX_C_166</t>
+  </si>
+  <si>
+    <t>MX_C_165</t>
+  </si>
+  <si>
+    <t>MX_C_164</t>
+  </si>
+  <si>
+    <t>MX_C_163</t>
+  </si>
+  <si>
+    <t>MX_C_158</t>
+  </si>
+  <si>
+    <t>MX_C_155</t>
+  </si>
+  <si>
+    <t>MX_C_154</t>
+  </si>
+  <si>
+    <t>MX_C_153</t>
+  </si>
+  <si>
+    <t>MX_C_151</t>
+  </si>
+  <si>
+    <t>MX_C_093</t>
+  </si>
+  <si>
+    <t>MX_C_150</t>
+  </si>
+  <si>
+    <t>MX_C_147</t>
+  </si>
+  <si>
+    <t>MX_C_145</t>
+  </si>
+  <si>
+    <t>MX_C_144</t>
+  </si>
+  <si>
+    <t>MX_C_143</t>
+  </si>
+  <si>
+    <t>MX_C_142</t>
+  </si>
+  <si>
+    <t>MX_C_140</t>
+  </si>
+  <si>
+    <t>MX_C_139</t>
+  </si>
+  <si>
+    <t>MX_C_136</t>
+  </si>
+  <si>
+    <t>MX_C_135</t>
+  </si>
+  <si>
+    <t>MX_C_092</t>
+  </si>
+  <si>
+    <t>MX_C_134</t>
+  </si>
+  <si>
+    <t>MX_C_130</t>
+  </si>
+  <si>
+    <t>MX_C_129</t>
+  </si>
+  <si>
+    <t>MX_C_128</t>
+  </si>
+  <si>
+    <t>MX_C_127</t>
+  </si>
+  <si>
+    <t>MX_C_125</t>
+  </si>
+  <si>
+    <t>MX_C_124</t>
+  </si>
+  <si>
+    <t>MX_C_123</t>
+  </si>
+  <si>
+    <t>MX_C_122</t>
+  </si>
+  <si>
+    <t>MX_C_121</t>
+  </si>
+  <si>
+    <t>MX_C_091</t>
+  </si>
+  <si>
+    <t>MX_C_120</t>
+  </si>
+  <si>
+    <t>MX_C_119</t>
+  </si>
+  <si>
+    <t>MX_C_118</t>
+  </si>
+  <si>
+    <t>MX_C_117</t>
+  </si>
+  <si>
+    <t>MX_C_116</t>
+  </si>
+  <si>
+    <t>MX_C_115</t>
+  </si>
+  <si>
+    <t>MX_C_114</t>
+  </si>
+  <si>
+    <t>MX_C_113</t>
+  </si>
+  <si>
+    <t>MX_C_112</t>
+  </si>
+  <si>
+    <t>MX_C_110</t>
+  </si>
+  <si>
+    <t>MX_C_090</t>
+  </si>
+  <si>
+    <t>MX_C_109</t>
+  </si>
+  <si>
+    <t>MX_C_108</t>
+  </si>
+  <si>
+    <t>MX_C_107</t>
+  </si>
+  <si>
+    <t>MX_C_106</t>
+  </si>
+  <si>
+    <t>MX_C_105</t>
+  </si>
+  <si>
+    <t>MX_C_104</t>
+  </si>
+  <si>
+    <t>MX_C_103</t>
+  </si>
+  <si>
+    <t>MX_C_102</t>
+  </si>
+  <si>
+    <t>MX_C_100</t>
+  </si>
+  <si>
+    <t>MX_C_192</t>
+  </si>
+  <si>
+    <t>MX_C_126</t>
+  </si>
+  <si>
+    <t>MX_C_191</t>
+  </si>
+  <si>
+    <t>MX_C_190</t>
+  </si>
+  <si>
+    <t>MX_C_149</t>
+  </si>
+  <si>
+    <t>MX_C_148</t>
+  </si>
+  <si>
+    <t>MX_C_146</t>
+  </si>
+  <si>
+    <t>MX_C_138</t>
+  </si>
+  <si>
+    <t>MX_C_137</t>
+  </si>
+  <si>
+    <t>MX_C_132</t>
+  </si>
+  <si>
+    <t>CAMARON</t>
+  </si>
+  <si>
+    <t>MX_C_195</t>
+  </si>
+  <si>
+    <t>MX_C_206</t>
+  </si>
+  <si>
+    <t>MX_C_204</t>
+  </si>
+  <si>
+    <t>Penaeus vannamei</t>
+  </si>
+  <si>
+    <t>CAMARON BLANCO</t>
+  </si>
+  <si>
+    <t>MX_C_012</t>
+  </si>
+  <si>
+    <t>ERIZO ROJO</t>
+  </si>
+  <si>
+    <t>MX_C_010</t>
+  </si>
+  <si>
+    <t>ERIZO MORADO</t>
+  </si>
+  <si>
+    <t>ALMEJA PISMO</t>
+  </si>
+  <si>
+    <t>MX_C_008</t>
+  </si>
+  <si>
+    <t>ALMEJA PATA DE MULA</t>
+  </si>
+  <si>
+    <t>MX_C_011</t>
+  </si>
+  <si>
+    <t>NODATA</t>
+  </si>
+  <si>
+    <t>MX_C_017</t>
+  </si>
+  <si>
+    <t>MX_C_212</t>
+  </si>
+  <si>
+    <t>MX_C_020</t>
+  </si>
+  <si>
+    <t>CARACOL PANOCHA</t>
+  </si>
+  <si>
+    <t>CANGREJO</t>
+  </si>
+  <si>
+    <t>PEPINO DE MAR</t>
+  </si>
+  <si>
+    <t>MX_C_006</t>
+  </si>
+  <si>
+    <t>PULPO</t>
+  </si>
+  <si>
+    <t>MX_C_030</t>
+  </si>
+  <si>
+    <t>ESCAMA ESTUARINA</t>
+  </si>
+  <si>
+    <t>ESCAMA GENERAL</t>
+  </si>
+  <si>
+    <t>MX_C_198</t>
+  </si>
+  <si>
+    <t>OSTION</t>
+  </si>
+  <si>
+    <t>Haliotis fulgens</t>
+  </si>
+  <si>
+    <t>Melongena patula</t>
+  </si>
+  <si>
+    <t>Panulirus interruptus</t>
+  </si>
+  <si>
+    <t>Strongylocentrotus purpuratus</t>
+  </si>
+  <si>
+    <t>Tivela stultorum</t>
+  </si>
+  <si>
+    <t>Callinectes spp.</t>
+  </si>
+  <si>
+    <t>Blue Land Crab</t>
+  </si>
+  <si>
+    <t>Swimming Crab</t>
+  </si>
+  <si>
+    <t>Rock Oyster</t>
+  </si>
+  <si>
+    <t>Red Algae</t>
+  </si>
+  <si>
+    <t>Pink Abalone</t>
+  </si>
+  <si>
+    <t>Green Abalone</t>
+  </si>
+  <si>
+    <t>Blue Shrimp</t>
+  </si>
+  <si>
+    <t>Bigclaw River Shrimp</t>
+  </si>
+  <si>
+    <t>Pacific Crown Conch</t>
+  </si>
+  <si>
+    <t>California Spiny Lobster</t>
+  </si>
+  <si>
+    <t>Caribbean Spiny Lobster</t>
+  </si>
+  <si>
+    <t>Green Spiny Lobster</t>
+  </si>
+  <si>
+    <t>Blue Spiny Lobster</t>
+  </si>
+  <si>
+    <t>Lobster</t>
+  </si>
+  <si>
+    <t>Brown Shrimp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shrimp </t>
+  </si>
+  <si>
+    <t>Pacific White Shrimp</t>
+  </si>
+  <si>
+    <t>Red Sea Urchin</t>
+  </si>
+  <si>
+    <t>Purple Sea Urchin</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Pismo Clam</t>
+  </si>
+  <si>
+    <t>Megastraea undosa</t>
+  </si>
+  <si>
+    <t>Anadara tuberculosa</t>
+  </si>
+  <si>
+    <t>Octopus vulgaris</t>
+  </si>
+  <si>
+    <t>Black Ark Clam</t>
+  </si>
+  <si>
+    <t>Wavy Turban Snail</t>
+  </si>
+  <si>
+    <t>Sea Cucumber</t>
+  </si>
+  <si>
+    <t>Common Octopus</t>
+  </si>
+  <si>
+    <t>Striostrea prismatica</t>
+  </si>
+  <si>
+    <t>unaccepted name originally  "litopenaeus stylirostris"</t>
+  </si>
+  <si>
+    <t>exclude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">where they are </t>
+  </si>
+  <si>
+    <t xml:space="preserve">exclude </t>
+  </si>
+  <si>
+    <t>Callinectes sapidus + Calinectes rathbunae</t>
+  </si>
+  <si>
+    <t>ERE PDFS INFO</t>
+  </si>
+  <si>
+    <t>Haliotis cracherodii</t>
+  </si>
+  <si>
+    <t>Black Abalone</t>
+  </si>
+  <si>
+    <t>Haliotis rufescens</t>
+  </si>
+  <si>
+    <t>Red Abalone</t>
+  </si>
+  <si>
+    <t>Haliotis sorenseni</t>
+  </si>
+  <si>
+    <t>White Abalone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eastern Oyster </t>
+  </si>
+  <si>
+    <t>Apostichopus parvimensis</t>
+  </si>
+  <si>
+    <t>Warty Sea Cucumber</t>
+  </si>
+  <si>
+    <t>Holothuria (Cystipus) inhabilis</t>
+  </si>
+  <si>
+    <t>White Sea Cucumber</t>
+  </si>
+  <si>
+    <t>Holothuria (Thymiosycia) impatiens</t>
+  </si>
+  <si>
+    <t>Mesocentrotus franciscanus</t>
+  </si>
+  <si>
+    <t>Penaeus stylirostris</t>
+  </si>
+  <si>
     <t>OSTION AMERICANO</t>
-  </si>
-  <si>
-    <t>MX_C_196</t>
-  </si>
-  <si>
-    <t>MX_C_193</t>
-  </si>
-  <si>
-    <t>MX_C_203</t>
-  </si>
-  <si>
-    <t>MX_C_209</t>
-  </si>
-  <si>
-    <t>MX_C_205</t>
-  </si>
-  <si>
-    <t>MX_C_052</t>
-  </si>
-  <si>
-    <t>Gelidium</t>
-  </si>
-  <si>
-    <t>ALGAS MARINAS</t>
-  </si>
-  <si>
-    <t>MX_C_007</t>
-  </si>
-  <si>
-    <t>Gelidium robustum</t>
-  </si>
-  <si>
-    <t>SARGAZO ROJO</t>
-  </si>
-  <si>
-    <t>MX_C_018</t>
-  </si>
-  <si>
-    <t>MX_C_031</t>
-  </si>
-  <si>
-    <t>MX_C_032</t>
-  </si>
-  <si>
-    <t>MX_C_024</t>
-  </si>
-  <si>
-    <t>Haliotis corrugata</t>
-  </si>
-  <si>
-    <t>ABULON AMARILLO</t>
-  </si>
-  <si>
-    <t>ABULON AZUL</t>
-  </si>
-  <si>
-    <t>MX_C_009</t>
-  </si>
-  <si>
-    <t>Haliotis spp.</t>
-  </si>
-  <si>
-    <t>ABULON</t>
-  </si>
-  <si>
-    <t>MX_C_025</t>
-  </si>
-  <si>
-    <t>MX_C_029</t>
-  </si>
-  <si>
-    <t>MX_C_041</t>
-  </si>
-  <si>
-    <t>Litopenaeus stylirostris</t>
-  </si>
-  <si>
-    <t>CAMARON AZUL</t>
-  </si>
-  <si>
-    <t>MX_C_037</t>
-  </si>
-  <si>
-    <t>MX_C_003</t>
-  </si>
-  <si>
-    <t>MX_C_051</t>
-  </si>
-  <si>
-    <t>MX_C_047</t>
-  </si>
-  <si>
-    <t>Macrobrachium carcinus</t>
-  </si>
-  <si>
-    <t>LANGOSTINO</t>
-  </si>
-  <si>
-    <t>Macrobrachium spp.</t>
-  </si>
-  <si>
-    <t>ACAMAYA</t>
-  </si>
-  <si>
-    <t>CARACOL BURRO</t>
-  </si>
-  <si>
-    <t>LANGOSTA ROJA</t>
-  </si>
-  <si>
-    <t>MX_C_066</t>
-  </si>
-  <si>
-    <t>Panulirus argus</t>
-  </si>
-  <si>
-    <t>LANGOSTA DEL CARIBE</t>
-  </si>
-  <si>
-    <t>MX_C_065</t>
-  </si>
-  <si>
-    <t>MX_C_068</t>
-  </si>
-  <si>
-    <t>MX_C_067</t>
-  </si>
-  <si>
-    <t>MX_C_064</t>
-  </si>
-  <si>
-    <t>MX_C_063</t>
-  </si>
-  <si>
-    <t>MX_C_062</t>
-  </si>
-  <si>
-    <t>MX_C_061</t>
-  </si>
-  <si>
-    <t>MX_C_217</t>
-  </si>
-  <si>
-    <t>MX_C_216</t>
-  </si>
-  <si>
-    <t>MX_C_215</t>
-  </si>
-  <si>
-    <t>MX_C_214</t>
-  </si>
-  <si>
-    <t>MX_C_213</t>
-  </si>
-  <si>
-    <t>Panulirus gracilis</t>
-  </si>
-  <si>
-    <t>LANGOSTA VERDE</t>
-  </si>
-  <si>
-    <t>Panulirus inflatus</t>
-  </si>
-  <si>
-    <t>LANGOSTA AZUL</t>
-  </si>
-  <si>
-    <t>Panulirus spp.</t>
-  </si>
-  <si>
-    <t>LANGOSTA</t>
-  </si>
-  <si>
-    <t>Penaeus aztecus</t>
-  </si>
-  <si>
-    <t>CAMARON CAFE</t>
-  </si>
-  <si>
-    <t>MX_C_039</t>
-  </si>
-  <si>
-    <t>MX_C_002</t>
-  </si>
-  <si>
-    <t>Penaeus spp.</t>
-  </si>
-  <si>
-    <t>CAMARON DE ESTERO</t>
-  </si>
-  <si>
-    <t>MX_C_057</t>
-  </si>
-  <si>
-    <t>MX_C_046</t>
-  </si>
-  <si>
-    <t>MX_C_045</t>
-  </si>
-  <si>
-    <t>MX_C_044</t>
-  </si>
-  <si>
-    <t>MX_C_043</t>
-  </si>
-  <si>
-    <t>MX_C_004</t>
-  </si>
-  <si>
-    <t>MX_C_055</t>
-  </si>
-  <si>
-    <t>MX_C_036</t>
-  </si>
-  <si>
-    <t>MX_C_035</t>
-  </si>
-  <si>
-    <t>MX_C_034</t>
-  </si>
-  <si>
-    <t>MX_C_033</t>
-  </si>
-  <si>
-    <t>MX_C_040</t>
-  </si>
-  <si>
-    <t>MX_C_054</t>
-  </si>
-  <si>
-    <t>MX_C_050</t>
-  </si>
-  <si>
-    <t>MX_C_098</t>
-  </si>
-  <si>
-    <t>MX_C_089</t>
-  </si>
-  <si>
-    <t>MX_C_088</t>
-  </si>
-  <si>
-    <t>MX_C_086</t>
-  </si>
-  <si>
-    <t>MX_C_085</t>
-  </si>
-  <si>
-    <t>MX_C_083</t>
-  </si>
-  <si>
-    <t>MX_C_082</t>
-  </si>
-  <si>
-    <t>MX_C_081</t>
-  </si>
-  <si>
-    <t>MX_C_080</t>
-  </si>
-  <si>
-    <t>MX_C_078</t>
-  </si>
-  <si>
-    <t>MX_C_097</t>
-  </si>
-  <si>
-    <t>MX_C_076</t>
-  </si>
-  <si>
-    <t>MX_C_075</t>
-  </si>
-  <si>
-    <t>MX_C_074</t>
-  </si>
-  <si>
-    <t>MX_C_073</t>
-  </si>
-  <si>
-    <t>MX_C_072</t>
-  </si>
-  <si>
-    <t>MX_C_071</t>
-  </si>
-  <si>
-    <t>MX_C_070</t>
-  </si>
-  <si>
-    <t>MX_C_069</t>
-  </si>
-  <si>
-    <t>MX_C_189</t>
-  </si>
-  <si>
-    <t>MX_C_188</t>
-  </si>
-  <si>
-    <t>MX_C_096</t>
-  </si>
-  <si>
-    <t>MX_C_187</t>
-  </si>
-  <si>
-    <t>MX_C_186</t>
-  </si>
-  <si>
-    <t>MX_C_185</t>
-  </si>
-  <si>
-    <t>MX_C_184</t>
-  </si>
-  <si>
-    <t>MX_C_183</t>
-  </si>
-  <si>
-    <t>MX_C_182</t>
-  </si>
-  <si>
-    <t>MX_C_181</t>
-  </si>
-  <si>
-    <t>MX_C_180</t>
-  </si>
-  <si>
-    <t>MX_C_179</t>
-  </si>
-  <si>
-    <t>MX_C_178</t>
-  </si>
-  <si>
-    <t>MX_C_095</t>
-  </si>
-  <si>
-    <t>MX_C_177</t>
-  </si>
-  <si>
-    <t>MX_C_176</t>
-  </si>
-  <si>
-    <t>MX_C_175</t>
-  </si>
-  <si>
-    <t>MX_C_174</t>
-  </si>
-  <si>
-    <t>MX_C_173</t>
-  </si>
-  <si>
-    <t>MX_C_172</t>
-  </si>
-  <si>
-    <t>MX_C_171</t>
-  </si>
-  <si>
-    <t>MX_C_170</t>
-  </si>
-  <si>
-    <t>MX_C_169</t>
-  </si>
-  <si>
-    <t>MX_C_168</t>
-  </si>
-  <si>
-    <t>MX_C_094</t>
-  </si>
-  <si>
-    <t>MX_C_167</t>
-  </si>
-  <si>
-    <t>MX_C_166</t>
-  </si>
-  <si>
-    <t>MX_C_165</t>
-  </si>
-  <si>
-    <t>MX_C_164</t>
-  </si>
-  <si>
-    <t>MX_C_163</t>
-  </si>
-  <si>
-    <t>MX_C_158</t>
-  </si>
-  <si>
-    <t>MX_C_155</t>
-  </si>
-  <si>
-    <t>MX_C_154</t>
-  </si>
-  <si>
-    <t>MX_C_153</t>
-  </si>
-  <si>
-    <t>MX_C_151</t>
-  </si>
-  <si>
-    <t>MX_C_093</t>
-  </si>
-  <si>
-    <t>MX_C_150</t>
-  </si>
-  <si>
-    <t>MX_C_147</t>
-  </si>
-  <si>
-    <t>MX_C_145</t>
-  </si>
-  <si>
-    <t>MX_C_144</t>
-  </si>
-  <si>
-    <t>MX_C_143</t>
-  </si>
-  <si>
-    <t>MX_C_142</t>
-  </si>
-  <si>
-    <t>MX_C_140</t>
-  </si>
-  <si>
-    <t>MX_C_139</t>
-  </si>
-  <si>
-    <t>MX_C_136</t>
-  </si>
-  <si>
-    <t>MX_C_135</t>
-  </si>
-  <si>
-    <t>MX_C_092</t>
-  </si>
-  <si>
-    <t>MX_C_134</t>
-  </si>
-  <si>
-    <t>MX_C_130</t>
-  </si>
-  <si>
-    <t>MX_C_129</t>
-  </si>
-  <si>
-    <t>MX_C_128</t>
-  </si>
-  <si>
-    <t>MX_C_127</t>
-  </si>
-  <si>
-    <t>MX_C_125</t>
-  </si>
-  <si>
-    <t>MX_C_124</t>
-  </si>
-  <si>
-    <t>MX_C_123</t>
-  </si>
-  <si>
-    <t>MX_C_122</t>
-  </si>
-  <si>
-    <t>MX_C_121</t>
-  </si>
-  <si>
-    <t>MX_C_091</t>
-  </si>
-  <si>
-    <t>MX_C_120</t>
-  </si>
-  <si>
-    <t>MX_C_119</t>
-  </si>
-  <si>
-    <t>MX_C_118</t>
-  </si>
-  <si>
-    <t>MX_C_117</t>
-  </si>
-  <si>
-    <t>MX_C_116</t>
-  </si>
-  <si>
-    <t>MX_C_115</t>
-  </si>
-  <si>
-    <t>MX_C_114</t>
-  </si>
-  <si>
-    <t>MX_C_113</t>
-  </si>
-  <si>
-    <t>MX_C_112</t>
-  </si>
-  <si>
-    <t>MX_C_110</t>
-  </si>
-  <si>
-    <t>MX_C_090</t>
-  </si>
-  <si>
-    <t>MX_C_109</t>
-  </si>
-  <si>
-    <t>MX_C_108</t>
-  </si>
-  <si>
-    <t>MX_C_107</t>
-  </si>
-  <si>
-    <t>MX_C_106</t>
-  </si>
-  <si>
-    <t>MX_C_105</t>
-  </si>
-  <si>
-    <t>MX_C_104</t>
-  </si>
-  <si>
-    <t>MX_C_103</t>
-  </si>
-  <si>
-    <t>MX_C_102</t>
-  </si>
-  <si>
-    <t>MX_C_100</t>
-  </si>
-  <si>
-    <t>MX_C_192</t>
-  </si>
-  <si>
-    <t>MX_C_126</t>
-  </si>
-  <si>
-    <t>MX_C_191</t>
-  </si>
-  <si>
-    <t>MX_C_190</t>
-  </si>
-  <si>
-    <t>MX_C_149</t>
-  </si>
-  <si>
-    <t>MX_C_148</t>
-  </si>
-  <si>
-    <t>MX_C_146</t>
-  </si>
-  <si>
-    <t>MX_C_138</t>
-  </si>
-  <si>
-    <t>MX_C_137</t>
-  </si>
-  <si>
-    <t>MX_C_132</t>
-  </si>
-  <si>
-    <t>CAMARON</t>
-  </si>
-  <si>
-    <t>MX_C_195</t>
-  </si>
-  <si>
-    <t>MX_C_206</t>
-  </si>
-  <si>
-    <t>MX_C_204</t>
-  </si>
-  <si>
-    <t>Penaeus vannamei</t>
-  </si>
-  <si>
-    <t>CAMARON BLANCO</t>
-  </si>
-  <si>
-    <t>MX_C_012</t>
-  </si>
-  <si>
-    <t>ERIZO ROJO</t>
-  </si>
-  <si>
-    <t>MX_C_010</t>
-  </si>
-  <si>
-    <t>ERIZO MORADO</t>
-  </si>
-  <si>
-    <t>ALMEJA PISMO</t>
-  </si>
-  <si>
-    <t>MX_C_008</t>
-  </si>
-  <si>
-    <t>ALMEJA PATA DE MULA</t>
-  </si>
-  <si>
-    <t>MX_C_011</t>
-  </si>
-  <si>
-    <t>NODATA</t>
-  </si>
-  <si>
-    <t>MX_C_017</t>
-  </si>
-  <si>
-    <t>MX_C_212</t>
-  </si>
-  <si>
-    <t>MX_C_020</t>
-  </si>
-  <si>
-    <t>CARACOL PANOCHA</t>
-  </si>
-  <si>
-    <t>CANGREJO</t>
-  </si>
-  <si>
-    <t>PEPINO DE MAR</t>
-  </si>
-  <si>
-    <t>MX_C_006</t>
-  </si>
-  <si>
-    <t>PULPO</t>
-  </si>
-  <si>
-    <t>MX_C_030</t>
-  </si>
-  <si>
-    <t>ESCAMA ESTUARINA</t>
-  </si>
-  <si>
-    <t>ESCAMA GENERAL</t>
-  </si>
-  <si>
-    <t>MX_C_198</t>
-  </si>
-  <si>
-    <t>OSTION</t>
-  </si>
-  <si>
-    <t>Haliotis fulgens</t>
-  </si>
-  <si>
-    <t>Melongena patula</t>
-  </si>
-  <si>
-    <t>Panulirus interruptus</t>
-  </si>
-  <si>
-    <t>Strongylocentrotus franciscanus</t>
-  </si>
-  <si>
-    <t>Strongylocentrotus purpuratus</t>
-  </si>
-  <si>
-    <t>Tivela stultorum</t>
-  </si>
-  <si>
-    <t>Callinectes spp.</t>
-  </si>
-  <si>
-    <t>Blue Land Crab</t>
-  </si>
-  <si>
-    <t>Swimming Crab</t>
-  </si>
-  <si>
-    <t>Rock Oyster</t>
-  </si>
-  <si>
-    <t>Eastern Osyter</t>
-  </si>
-  <si>
-    <t>Red Algae</t>
-  </si>
-  <si>
-    <t>Pink Abalone</t>
-  </si>
-  <si>
-    <t>Green Abalone</t>
-  </si>
-  <si>
-    <t>Abalone</t>
-  </si>
-  <si>
-    <t>Blue Shrimp</t>
-  </si>
-  <si>
-    <t>Bigclaw River Shrimp</t>
-  </si>
-  <si>
-    <t>Freshwater Shrimp</t>
-  </si>
-  <si>
-    <t>Pacific Crown Conch</t>
-  </si>
-  <si>
-    <t>California Spiny Lobster</t>
-  </si>
-  <si>
-    <t>Caribbean Spiny Lobster</t>
-  </si>
-  <si>
-    <t>Green Spiny Lobster</t>
-  </si>
-  <si>
-    <t>Blue Spiny Lobster</t>
-  </si>
-  <si>
-    <t>Lobster</t>
-  </si>
-  <si>
-    <t>Brown Shrimp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shrimp </t>
-  </si>
-  <si>
-    <t>Pacific White Shrimp</t>
-  </si>
-  <si>
-    <t>Red Sea Urchin</t>
-  </si>
-  <si>
-    <t>Purple Sea Urchin</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Pismo Clam</t>
-  </si>
-  <si>
-    <t>Megastraea undosa</t>
-  </si>
-  <si>
-    <t>Anadara tuberculosa</t>
-  </si>
-  <si>
-    <t>Holothuroidea</t>
-  </si>
-  <si>
-    <t>Octopus vulgaris</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crassostrea </t>
-  </si>
-  <si>
-    <t>Black Ark Clam</t>
-  </si>
-  <si>
-    <t>Wavy Turban Snail</t>
-  </si>
-  <si>
-    <t>Sea Cucumber</t>
-  </si>
-  <si>
-    <t>Common Octopus</t>
-  </si>
-  <si>
-    <t>Oyster</t>
-  </si>
-  <si>
-    <t>Striostrea prismatica</t>
-  </si>
-  <si>
-    <t>unaccepted name originally  "litopenaeus stylirostris"</t>
-  </si>
-  <si>
-    <t>exclude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">where they are </t>
-  </si>
-  <si>
-    <t xml:space="preserve">exclude </t>
-  </si>
-  <si>
-    <t>Callinectes sapidus + Calinectes rathbunae</t>
-  </si>
-  <si>
-    <t>ERE PDFS INFO</t>
   </si>
 </sst>
 </file>
@@ -1352,7 +1364,9 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1761,7 +1775,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
@@ -1769,13 +1783,13 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="E2">
         <v>106921</v>
@@ -1792,7 +1806,7 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="E3">
         <v>422183</v>
@@ -1803,19 +1817,19 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="C4" t="s">
         <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="E4">
         <v>506739</v>
       </c>
       <c r="F4" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
@@ -1823,19 +1837,19 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="E5">
-        <v>140657</v>
+        <v>144135</v>
       </c>
       <c r="F5" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
@@ -1843,16 +1857,16 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="E6">
-        <v>144135</v>
+        <v>372718</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
@@ -1860,16 +1874,16 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="E7">
-        <v>372718</v>
+        <v>445308</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
@@ -1877,16 +1891,16 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>229</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="E8">
-        <v>445308</v>
+        <v>445325</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
@@ -1894,335 +1908,335 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>233</v>
+        <v>282</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="E9">
-        <v>445325</v>
+        <v>584982</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>247</v>
+      <c r="B10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" t="s">
+        <v>242</v>
       </c>
       <c r="E10">
-        <v>138050</v>
+        <v>246169</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>248</v>
+      <c r="B11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" t="s">
+        <v>242</v>
       </c>
       <c r="E11">
-        <v>1809211</v>
+        <v>246169</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
+        <v>230</v>
+      </c>
+      <c r="C12" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>249</v>
+      <c r="D12" t="s">
+        <v>243</v>
       </c>
       <c r="E12">
-        <v>246169</v>
+        <v>567144</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>250</v>
+      <c r="B13" t="s">
+        <v>231</v>
+      </c>
+      <c r="C13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" t="s">
+        <v>244</v>
       </c>
       <c r="E13">
-        <v>156892</v>
+        <v>382898</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="C14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>251</v>
+      <c r="D14" t="s">
+        <v>245</v>
       </c>
       <c r="E14">
-        <v>567144</v>
+        <v>382891</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>22</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>252</v>
+        <v>21</v>
+      </c>
+      <c r="B15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" t="s">
+        <v>246</v>
       </c>
       <c r="E15">
-        <v>382898</v>
+        <v>382895</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>253</v>
+        <v>22</v>
+      </c>
+      <c r="B16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" t="s">
+        <v>247</v>
       </c>
       <c r="E16">
-        <v>382891</v>
+        <v>382897</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" t="s">
         <v>72</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" t="s">
         <v>73</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>254</v>
+      <c r="D17" t="s">
+        <v>248</v>
       </c>
       <c r="E17">
-        <v>382895</v>
+        <v>107060</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" t="s">
         <v>74</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" t="s">
         <v>75</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>255</v>
+      <c r="D18" t="s">
+        <v>249</v>
       </c>
       <c r="E18">
-        <v>382897</v>
+        <v>1809216</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>256</v>
+      <c r="B19" t="s">
+        <v>78</v>
+      </c>
+      <c r="C19" t="s">
+        <v>79</v>
+      </c>
+      <c r="D19" t="s">
+        <v>250</v>
       </c>
       <c r="E19">
-        <v>107060</v>
+        <v>106822</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>26</v>
-      </c>
-      <c r="B20" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" t="s">
         <v>78</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>257</v>
+      <c r="C20" t="s">
+        <v>201</v>
+      </c>
+      <c r="D20" t="s">
+        <v>250</v>
       </c>
       <c r="E20">
-        <v>1809216</v>
+        <v>106822</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>258</v>
+        <v>25</v>
+      </c>
+      <c r="B21" t="s">
+        <v>205</v>
+      </c>
+      <c r="C21" t="s">
+        <v>206</v>
+      </c>
+      <c r="D21" t="s">
+        <v>251</v>
       </c>
       <c r="E21">
-        <v>106822</v>
+        <v>1809212</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>258</v>
+        <v>25</v>
+      </c>
+      <c r="B22" t="s">
+        <v>281</v>
+      </c>
+      <c r="C22" t="s">
+        <v>208</v>
+      </c>
+      <c r="D22" t="s">
+        <v>252</v>
       </c>
       <c r="E22">
-        <v>106822</v>
+        <v>591102</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>26</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="C23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" t="s">
+        <v>232</v>
+      </c>
+      <c r="C23" t="s">
         <v>210</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>259</v>
+      <c r="D23" t="s">
+        <v>253</v>
       </c>
       <c r="E23">
-        <v>1809212</v>
+        <v>240747</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>29</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>260</v>
+        <v>28</v>
+      </c>
+      <c r="B24" t="s">
+        <v>233</v>
+      </c>
+      <c r="C24" t="s">
+        <v>211</v>
+      </c>
+      <c r="D24" t="s">
+        <v>254</v>
       </c>
       <c r="E24">
-        <v>240762</v>
+        <v>367761</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>261</v>
+        <v>28</v>
+      </c>
+      <c r="B25" t="s">
+        <v>256</v>
+      </c>
+      <c r="C25" t="s">
+        <v>213</v>
+      </c>
+      <c r="D25" t="s">
+        <v>258</v>
       </c>
       <c r="E25">
-        <v>240747</v>
+        <v>504313</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>29</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="C26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" t="s">
         <v>215</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="E26">
-        <v>367761</v>
+      <c r="D26" t="s">
+        <v>7</v>
+      </c>
+      <c r="E26" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>268</v>
+        <v>28</v>
+      </c>
+      <c r="B27" t="s">
+        <v>255</v>
+      </c>
+      <c r="C27" t="s">
+        <v>219</v>
+      </c>
+      <c r="D27" t="s">
+        <v>259</v>
       </c>
       <c r="E27">
-        <v>504313</v>
+        <v>528084</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="C28" t="s">
+        <v>220</v>
+      </c>
+      <c r="D28" t="s">
         <v>7</v>
       </c>
       <c r="E28" t="s">
@@ -2231,32 +2245,32 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>29</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="C29" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>257</v>
+      </c>
+      <c r="C29" t="s">
         <v>223</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>269</v>
+      <c r="D29" t="s">
+        <v>261</v>
       </c>
       <c r="E29">
-        <v>528084</v>
+        <v>140605</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>29</v>
-      </c>
-      <c r="B30" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="D30" s="2" t="s">
+      <c r="C30" t="s">
+        <v>225</v>
+      </c>
+      <c r="D30" t="s">
         <v>7</v>
       </c>
       <c r="E30" t="s">
@@ -2265,180 +2279,249 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>29</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="E31">
-        <v>123083</v>
+        <v>28</v>
+      </c>
+      <c r="B31" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" t="s">
+        <v>226</v>
+      </c>
+      <c r="D31" t="s">
+        <v>7</v>
+      </c>
+      <c r="E31" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>29</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>271</v>
+        <v>28</v>
+      </c>
+      <c r="B32" t="s">
+        <v>269</v>
+      </c>
+      <c r="C32" t="s">
+        <v>39</v>
+      </c>
+      <c r="D32" t="s">
+        <v>270</v>
       </c>
       <c r="E32">
-        <v>140605</v>
+        <v>405012</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>29</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E33" t="s">
-        <v>7</v>
+        <v>28</v>
+      </c>
+      <c r="B33" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" t="s">
+        <v>39</v>
+      </c>
+      <c r="D33" t="s">
+        <v>239</v>
+      </c>
+      <c r="E33">
+        <v>445308</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>29</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E34" t="s">
-        <v>7</v>
+        <v>28</v>
+      </c>
+      <c r="B34" t="s">
+        <v>229</v>
+      </c>
+      <c r="C34" t="s">
+        <v>39</v>
+      </c>
+      <c r="D34" t="s">
+        <v>240</v>
+      </c>
+      <c r="E34">
+        <v>445325</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>29</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="D35" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B35" t="s">
+        <v>271</v>
+      </c>
+      <c r="C35" t="s">
+        <v>39</v>
+      </c>
+      <c r="D35" t="s">
         <v>272</v>
       </c>
       <c r="E35">
-        <v>138297</v>
+        <v>445357</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>29</v>
-      </c>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="B36" t="s">
+        <v>273</v>
+      </c>
+      <c r="C36" t="s">
+        <v>39</v>
+      </c>
+      <c r="D36" t="s">
+        <v>274</v>
+      </c>
+      <c r="E36">
+        <v>445362</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="B37" t="s">
+        <v>19</v>
+      </c>
+      <c r="C37" t="s">
+        <v>228</v>
+      </c>
+      <c r="D37" t="s">
+        <v>275</v>
+      </c>
+      <c r="E37">
+        <v>140657</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="E38" s="2">
+        <v>529435</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="E39" s="2">
+        <v>241825</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="E40" s="2">
+        <v>125185</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="E41" s="2">
+        <v>140657</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.45">
@@ -2448,50 +2531,50 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G59" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.45">
@@ -2504,7 +2587,7 @@
         <v>9</v>
       </c>
       <c r="G65" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.45">
@@ -2512,7 +2595,7 @@
         <v>10</v>
       </c>
       <c r="G66" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.45">
@@ -2522,7 +2605,7 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.45">
@@ -2532,67 +2615,67 @@
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.45">
@@ -2602,7 +2685,7 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.45">
@@ -2617,15 +2700,15 @@
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G87" s="1" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.45">
@@ -2635,127 +2718,127 @@
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.45">
@@ -2765,537 +2848,537 @@
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A164" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A165" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A166" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A167" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A168" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A169" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A170" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A171" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A172" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A173" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A174" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A175" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A176" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A177" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A178" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A179" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A180" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A181" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="182" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A182" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A183" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="184" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A184" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="185" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A185" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="186" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A186" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="187" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A187" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A188" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="189" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A189" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="190" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A190" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="191" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A191" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="192" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A192" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A193" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A194" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A195" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="196" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A196" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="197" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A197" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="198" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A198" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="199" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A199" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="200" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A200" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="201" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A201" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="202" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A202" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="203" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A203" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="204" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A204" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="205" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A205" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="206" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A206" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="207" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A207" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="208" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A208" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="209" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A209" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="210" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A210" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="211" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A211" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="212" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A212" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="213" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A213" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="214" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A214" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="215" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A215" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="216" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A216" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="217" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A217" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="218" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A218" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="219" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A219" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="220" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A220" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="221" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A221" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="222" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A222" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
     </row>
     <row r="223" spans="1:1" x14ac:dyDescent="0.45">
@@ -3310,22 +3393,22 @@
     </row>
     <row r="225" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A225" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="226" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A226" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="227" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A227" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="228" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A228" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="229" spans="1:1" x14ac:dyDescent="0.45">
@@ -3335,7 +3418,7 @@
     </row>
     <row r="230" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A230" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="231" spans="1:1" x14ac:dyDescent="0.45">
@@ -3345,12 +3428,12 @@
     </row>
     <row r="232" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A232" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
     </row>
     <row r="233" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A233" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
     </row>
     <row r="234" spans="1:1" x14ac:dyDescent="0.45">
@@ -3360,192 +3443,192 @@
     </row>
     <row r="235" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A235" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="236" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A236" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="237" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A237" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="238" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A238" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="239" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A239" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="240" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A240" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="241" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A241" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="242" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A242" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="243" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A243" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="244" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A244" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="245" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A245" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="246" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A246" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="247" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A247" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="248" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A248" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="249" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A249" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="250" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A250" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="251" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A251" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="252" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A252" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="253" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A253" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="254" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A254" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="255" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A255" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="256" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A256" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="257" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A257" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
     <row r="258" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A258" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="259" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A259" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="260" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A260" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="261" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A261" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="262" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A262" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="263" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A263" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="264" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A264" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="265" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A265" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="266" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A266" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="267" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A267" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="268" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A268" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="269" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A269" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="270" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A270" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="271" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A271" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="272" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A272" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="273" spans="1:1" x14ac:dyDescent="0.45">
@@ -3560,17 +3643,17 @@
     </row>
     <row r="275" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A275" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
     </row>
     <row r="276" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A276" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="277" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A277" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="278" spans="1:1" x14ac:dyDescent="0.45">
@@ -3580,7 +3663,7 @@
     </row>
     <row r="279" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A279" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="280" spans="1:1" x14ac:dyDescent="0.45">
@@ -3590,12 +3673,12 @@
     </row>
     <row r="281" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A281" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
     </row>
     <row r="282" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A282" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
     </row>
     <row r="283" spans="1:1" x14ac:dyDescent="0.45">

</xml_diff>